<commit_message>
latest code checked In
</commit_message>
<xml_diff>
--- a/system_info.xlsx
+++ b/system_info.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,12 +421,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -450,8 +438,8 @@
           <t>Date</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>46097</v>
+      <c r="B2" s="1" t="n">
+        <v>46099</v>
       </c>
     </row>
     <row r="3">
@@ -462,7 +450,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>192.168.31.235</t>
+          <t>192.168.1.14</t>
         </is>
       </c>
     </row>
@@ -474,7 +462,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Intel64 Family 6 Model 140 Stepping 2, GenuineIntel</t>
+          <t>Intel64 Family 6 Model 165 Stepping 2, GenuineIntel</t>
         </is>
       </c>
     </row>
@@ -510,7 +498,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dushyant</t>
+          <t>Alankrit</t>
         </is>
       </c>
     </row>

</xml_diff>